<commit_message>
modify generic synfuels to use market-average H2
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-ships.xlsx
+++ b/premise/data/additional_inventories/lci-ships.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/Github/premise/premise/data/additional_inventories/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romain/GitHub/premise/premise/data/additional_inventories/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF4F689-4E17-1741-A45E-48F2FB1E57CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F426A898-438A-DF44-8F37-3DD825F25669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20240" yWindow="720" windowWidth="22420" windowHeight="23000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10500" yWindow="660" windowWidth="25820" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="inventories" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="200">
   <si>
     <t>Database</t>
   </si>
@@ -209,9 +209,6 @@
     <t>transport, freight, sea, container ship, powered with liquid ammonia</t>
   </si>
   <si>
-    <t>ammonia production, hydrogen from electrolysis</t>
-  </si>
-  <si>
     <t>ammonia, anhydrous, liquid</t>
   </si>
   <si>
@@ -239,9 +236,6 @@
     <t>20% penalty of load carrying capacity, due to the low gravimetric density of methanol.</t>
   </si>
   <si>
-    <t>methanol distillation, hydrogen from electrolysis, CO2 from DAC</t>
-  </si>
-  <si>
     <t>methanol, purified</t>
   </si>
   <si>
@@ -383,9 +377,6 @@
     <t>Dinitrogen monoxide</t>
   </si>
   <si>
-    <t>liquefied petroleum gas production, from methanol, hydrogen from electrolysis, CO2 from DAC, energy allocation</t>
-  </si>
-  <si>
     <t>liquefied petroleum gas, synthetic</t>
   </si>
   <si>
@@ -542,9 +533,6 @@
     <t>Based on the ecoinvent dataset transport, freight, sea, container ship, to which we add an input of synthetic diesel and corresponding emissions. We assume a similar tank-to-wake efficiency as that of a martime oil-powered ship.</t>
   </si>
   <si>
-    <t>diesel production, synthetic, Fischer Tropsch process, hydrogen from electrolysis, energy allocation</t>
-  </si>
-  <si>
     <t>Assumes similar efficiency as with an oil-powered ship. Diesel LHV: 43 MJ/kg.</t>
   </si>
   <si>
@@ -627,6 +615,27 @@
   </si>
   <si>
     <t>80% reduction relative to using HFO at 75% engine load, according to Petzold et al., 2011, dx.doi.org/10.1021/es2021439</t>
+  </si>
+  <si>
+    <t>LPG (propane and butane)</t>
+  </si>
+  <si>
+    <t>26--27</t>
+  </si>
+  <si>
+    <t>9% penalty of load carrying capacity, due to the low gravimetric density of LPG.</t>
+  </si>
+  <si>
+    <t>diesel production, synthetic, Fischer Tropsch process, market-average hydrogen, energy allocation</t>
+  </si>
+  <si>
+    <t>liquefied petroleum gas production, from methanol, market-average hydrogen, CO2 from DAC, energy allocation</t>
+  </si>
+  <si>
+    <t>methanol distillation, market-average hydrogen, CO2 from DAC</t>
+  </si>
+  <si>
+    <t>ammonia production, with market-average hydrogen</t>
   </si>
 </sst>
 </file>
@@ -634,11 +643,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -701,7 +710,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
@@ -709,12 +718,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -723,17 +732,17 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1076,7 +1085,7 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -1084,7 +1093,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -1113,7 +1122,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B10">
         <f>parameters!N7</f>
@@ -1122,7 +1131,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B11">
         <f>parameters!O7</f>
@@ -1131,7 +1140,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B12">
         <f>parameters!P7</f>
@@ -1140,7 +1149,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B13" s="13">
         <f>parameters!I7</f>
@@ -1149,7 +1158,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B14" s="13">
         <f>parameters!J7</f>
@@ -1158,7 +1167,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B15" s="13">
         <f>parameters!K7</f>
@@ -1167,7 +1176,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B16" s="13">
         <f>parameters!$C$15</f>
@@ -1176,7 +1185,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B17" s="13">
         <f>parameters!C18</f>
@@ -1185,7 +1194,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B18" s="13">
         <f>parameters!D18</f>
@@ -1194,7 +1203,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B19" s="13">
         <f>parameters!E18</f>
@@ -1288,7 +1297,7 @@
         <v>41</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I23" s="5">
         <v>5</v>
@@ -1446,7 +1455,7 @@
         <v>43</v>
       </c>
       <c r="H27" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I27">
         <v>5</v>
@@ -1485,7 +1494,7 @@
         <v>49</v>
       </c>
       <c r="H28" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I28">
         <v>5</v>
@@ -1540,13 +1549,13 @@
         <v>23</v>
       </c>
       <c r="E30" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F30" t="s">
         <v>20</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J30" s="11"/>
       <c r="K30" s="11"/>
@@ -1568,7 +1577,7 @@
         <v>11</v>
       </c>
       <c r="B33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -1605,7 +1614,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B38" s="15">
         <f>parameters!N8</f>
@@ -1614,7 +1623,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B39" s="15">
         <f>parameters!O8</f>
@@ -1623,7 +1632,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B40">
         <f>parameters!P8</f>
@@ -1632,7 +1641,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B41" s="13">
         <f>parameters!I8</f>
@@ -1641,7 +1650,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B42" s="13">
         <f>parameters!J8</f>
@@ -1650,7 +1659,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B43" s="13">
         <f>parameters!K8</f>
@@ -1659,7 +1668,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B44" s="13">
         <f>parameters!$C$15</f>
@@ -1668,7 +1677,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B45" s="13">
         <f>parameters!C19</f>
@@ -1677,7 +1686,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B46" s="13">
         <f>parameters!D19</f>
@@ -1686,7 +1695,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B47" s="13">
         <f>parameters!E19</f>
@@ -1761,7 +1770,7 @@
     </row>
     <row r="51" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B51" s="17">
         <f>0.11*(B44/B45)/3.6/(1-B41)</f>
@@ -1780,7 +1789,7 @@
         <v>22</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I51">
         <v>5</v>
@@ -1952,7 +1961,7 @@
         <v>11</v>
       </c>
       <c r="B58" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
@@ -1960,7 +1969,7 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
@@ -1989,7 +1998,7 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B63">
         <f>parameters!N6</f>
@@ -1998,7 +2007,7 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B64">
         <f>parameters!O6</f>
@@ -2007,7 +2016,7 @@
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B65">
         <f>parameters!P6</f>
@@ -2016,7 +2025,7 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B66" s="13">
         <f>parameters!I6</f>
@@ -2025,7 +2034,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B67" s="13">
         <f>parameters!J6</f>
@@ -2034,7 +2043,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B68" s="13">
         <f>parameters!K6</f>
@@ -2043,7 +2052,7 @@
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B69" s="13">
         <f>parameters!$C$15</f>
@@ -2052,7 +2061,7 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B70" s="13">
         <f>parameters!C17</f>
@@ -2061,7 +2070,7 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B71" s="13">
         <f>parameters!D17</f>
@@ -2070,7 +2079,7 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B72" s="13">
         <f>parameters!E17</f>
@@ -2145,7 +2154,7 @@
     </row>
     <row r="76" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>57</v>
+        <v>199</v>
       </c>
       <c r="B76" s="12">
         <f>(0.11*(B69/B70))/18.6/(1-B66)</f>
@@ -2161,10 +2170,10 @@
         <v>17</v>
       </c>
       <c r="G76" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H76" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I76">
         <v>5</v>
@@ -2203,7 +2212,7 @@
         <v>32</v>
       </c>
       <c r="H77" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I77">
         <v>5</v>
@@ -2242,7 +2251,7 @@
         <v>43</v>
       </c>
       <c r="H78" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I78">
         <v>5</v>
@@ -2281,7 +2290,7 @@
         <v>49</v>
       </c>
       <c r="H79" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I79">
         <v>5</v>
@@ -2325,7 +2334,7 @@
     </row>
     <row r="81" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B81">
         <f>0.00013*(B76*18.6*B70/3.6)</f>
@@ -2341,7 +2350,7 @@
         <v>20</v>
       </c>
       <c r="H81" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I81">
         <v>5</v>
@@ -2377,7 +2386,7 @@
         <v>20</v>
       </c>
       <c r="H82" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I82">
         <v>5</v>
@@ -2397,7 +2406,7 @@
     </row>
     <row r="83" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B83">
         <f>0.00002*(B76*18.6*B70/3.6)</f>
@@ -2413,7 +2422,7 @@
         <v>20</v>
       </c>
       <c r="H83" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I83">
         <v>5</v>
@@ -2433,7 +2442,7 @@
     </row>
     <row r="84" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B84">
         <f>0.0000028*(B76*18.6*B70/3.6)</f>
@@ -2449,7 +2458,7 @@
         <v>20</v>
       </c>
       <c r="H84" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I84">
         <v>5</v>
@@ -2485,7 +2494,7 @@
         <v>20</v>
       </c>
       <c r="H85" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I85">
         <v>5</v>
@@ -2505,7 +2514,7 @@
     </row>
     <row r="86" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B86">
         <f>0.000046*(B76*18.6*B70/3.6)</f>
@@ -2521,7 +2530,7 @@
         <v>20</v>
       </c>
       <c r="H86" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I86">
         <v>5</v>
@@ -2548,7 +2557,7 @@
         <v>3</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.2">
@@ -2556,7 +2565,7 @@
         <v>11</v>
       </c>
       <c r="B89" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.2">
@@ -2564,7 +2573,7 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.2">
@@ -2593,7 +2602,7 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B94">
         <f>parameters!N5</f>
@@ -2602,7 +2611,7 @@
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B95">
         <f>parameters!O5</f>
@@ -2611,7 +2620,7 @@
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B96">
         <f>parameters!P5</f>
@@ -2620,7 +2629,7 @@
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B97" s="13">
         <f>parameters!I5</f>
@@ -2629,7 +2638,7 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B98" s="13">
         <f>parameters!J5</f>
@@ -2638,7 +2647,7 @@
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B99" s="13">
         <f>parameters!K5</f>
@@ -2647,7 +2656,7 @@
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B100" s="13">
         <f>parameters!$C$15</f>
@@ -2656,7 +2665,7 @@
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B101" s="13">
         <f>parameters!C16</f>
@@ -2665,7 +2674,7 @@
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B102" s="13">
         <f>parameters!D16</f>
@@ -2674,7 +2683,7 @@
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B103" s="13">
         <f>parameters!E16</f>
@@ -2749,7 +2758,7 @@
     </row>
     <row r="107" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>67</v>
+        <v>198</v>
       </c>
       <c r="B107" s="12">
         <f>0.11*(B100/B101)/19.9/(1-B97)</f>
@@ -2765,10 +2774,10 @@
         <v>17</v>
       </c>
       <c r="G107" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H107" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I107">
         <v>5</v>
@@ -2807,7 +2816,7 @@
         <v>43</v>
       </c>
       <c r="H108" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I108">
         <v>5</v>
@@ -2846,7 +2855,7 @@
         <v>49</v>
       </c>
       <c r="H109" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I109">
         <v>5</v>
@@ -2890,7 +2899,7 @@
     </row>
     <row r="111" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B111" s="12">
         <f>B107*1.37</f>
@@ -2906,7 +2915,7 @@
         <v>20</v>
       </c>
       <c r="H111" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I111">
         <v>5</v>
@@ -2926,7 +2935,7 @@
     </row>
     <row r="112" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B112" s="11">
         <f>0.0048*(B107*19.9*B101/3.6)</f>
@@ -2942,7 +2951,7 @@
         <v>20</v>
       </c>
       <c r="H112" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I112">
         <v>5</v>
@@ -2978,7 +2987,7 @@
         <v>20</v>
       </c>
       <c r="H113" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I113">
         <v>5</v>
@@ -2998,7 +3007,7 @@
     </row>
     <row r="114" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B114">
         <f>0.00695*B107*0.9</f>
@@ -3014,7 +3023,7 @@
         <v>20</v>
       </c>
       <c r="H114" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="I114">
         <v>5</v>
@@ -3050,7 +3059,7 @@
         <v>20</v>
       </c>
       <c r="H115" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I115">
         <v>5</v>
@@ -3078,7 +3087,7 @@
         <v>3</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.2">
@@ -3086,7 +3095,7 @@
         <v>11</v>
       </c>
       <c r="B118" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.2">
@@ -3094,7 +3103,7 @@
         <v>10</v>
       </c>
       <c r="B119" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.2">
@@ -3123,7 +3132,7 @@
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B123" s="11">
         <f>parameters!N10</f>
@@ -3132,7 +3141,7 @@
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B124" s="11">
         <f>parameters!O10</f>
@@ -3141,7 +3150,7 @@
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B125" s="11">
         <f>parameters!P10</f>
@@ -3150,7 +3159,7 @@
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B126" s="13">
         <f>parameters!I10</f>
@@ -3159,7 +3168,7 @@
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B127" s="13">
         <f>parameters!J10</f>
@@ -3168,7 +3177,7 @@
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B128" s="13">
         <f>parameters!K10</f>
@@ -3177,7 +3186,7 @@
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B129" s="13">
         <f>parameters!$C$15</f>
@@ -3186,7 +3195,7 @@
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B130" s="13">
         <f>parameters!C21</f>
@@ -3195,7 +3204,7 @@
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B131" s="13">
         <f>parameters!D21</f>
@@ -3204,7 +3213,7 @@
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B132" s="13">
         <f>parameters!E21</f>
@@ -3279,7 +3288,7 @@
     </row>
     <row r="136" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B136" s="12">
         <f>0.11*(B129/B130)/47.5/(1-B126)</f>
@@ -3295,10 +3304,10 @@
         <v>17</v>
       </c>
       <c r="G136" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H136" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I136">
         <v>5</v>
@@ -3337,7 +3346,7 @@
         <v>43</v>
       </c>
       <c r="H137" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I137">
         <v>5</v>
@@ -3376,7 +3385,7 @@
         <v>49</v>
       </c>
       <c r="H138" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I138">
         <v>5</v>
@@ -3420,7 +3429,7 @@
     </row>
     <row r="140" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B140" s="12">
         <f>B136*2.74</f>
@@ -3436,7 +3445,7 @@
         <v>20</v>
       </c>
       <c r="H140" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I140">
         <v>5</v>
@@ -3456,7 +3465,7 @@
     </row>
     <row r="141" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B141" s="11">
         <f>0.00186*(B136*48*B130/3.6)</f>
@@ -3472,7 +3481,7 @@
         <v>20</v>
       </c>
       <c r="H141" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I141">
         <v>5</v>
@@ -3508,7 +3517,7 @@
         <v>20</v>
       </c>
       <c r="H142" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I142">
         <v>5</v>
@@ -3528,7 +3537,7 @@
     </row>
     <row r="143" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B143" s="11">
         <f>0.00003*(B136*48*B130/3.6)</f>
@@ -3544,7 +3553,7 @@
         <v>20</v>
       </c>
       <c r="H143" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I143">
         <v>5</v>
@@ -3564,7 +3573,7 @@
     </row>
     <row r="144" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B144" s="11">
         <f>0.00003*(B136*48*B130/3.6)</f>
@@ -3580,7 +3589,7 @@
         <v>20</v>
       </c>
       <c r="H144" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I144">
         <v>5</v>
@@ -3600,7 +3609,7 @@
     </row>
     <row r="145" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B145" s="11">
         <f>B136*0.02</f>
@@ -3616,7 +3625,7 @@
         <v>20</v>
       </c>
       <c r="H145" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I145">
         <v>5</v>
@@ -3636,7 +3645,7 @@
     </row>
     <row r="146" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B146" s="11">
         <f>0.00038*(B136*48*B130/3.6)</f>
@@ -3652,7 +3661,7 @@
         <v>20</v>
       </c>
       <c r="H146" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I146">
         <v>5</v>
@@ -3672,7 +3681,7 @@
     </row>
     <row r="147" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B147" s="11">
         <f>0.00002*(B136*48*B130/3.6)</f>
@@ -3688,7 +3697,7 @@
         <v>20</v>
       </c>
       <c r="H147" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I147">
         <v>5</v>
@@ -3711,7 +3720,7 @@
         <v>3</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.2">
@@ -3719,7 +3728,7 @@
         <v>11</v>
       </c>
       <c r="B151" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.2">
@@ -3727,7 +3736,7 @@
         <v>10</v>
       </c>
       <c r="B152" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.2">
@@ -3756,61 +3765,61 @@
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B156" s="11">
-        <f>parameters!N9</f>
-        <v>158400000000</v>
+        <f>parameters!N11</f>
+        <v>163923092656.98508</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B157" s="11">
-        <f>parameters!O9</f>
-        <v>153000000000</v>
+        <f>parameters!O11</f>
+        <v>159903865821.23132</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B158" s="11">
-        <f>parameters!P9</f>
-        <v>162000000000</v>
+        <f>parameters!P11</f>
+        <v>166602577214.15421</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B159" s="13">
-        <f>parameters!I9</f>
-        <v>0.12</v>
+        <f>parameters!I11</f>
+        <v>8.9316151905638519E-2</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B160" s="13">
-        <f>parameters!J9</f>
-        <v>0.1</v>
+        <f>parameters!J11</f>
+        <v>7.4430126588032122E-2</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B161" s="13">
-        <f>parameters!K9</f>
-        <v>0.15</v>
+        <f>parameters!K11</f>
+        <v>0.11164518988204816</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B162" s="13">
         <f>parameters!$C$15</f>
@@ -3819,28 +3828,28 @@
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B163" s="13">
-        <f>parameters!C20</f>
+        <f>parameters!C23</f>
         <v>0.49342105263157898</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B164" s="13">
-        <f>parameters!D20</f>
+        <f>parameters!D23</f>
         <v>0.44407894736842107</v>
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B165" s="13">
-        <f>parameters!E20</f>
+        <f>parameters!E23</f>
         <v>0.54276315789473695</v>
       </c>
     </row>
@@ -3912,11 +3921,11 @@
     </row>
     <row r="169" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>115</v>
+        <v>197</v>
       </c>
       <c r="B169" s="12">
         <f>0.11*(B162/B163)/46/(1-B159)</f>
-        <v>2.3405797101449274E-3</v>
+        <v>2.261718102541901E-3</v>
       </c>
       <c r="C169" t="s">
         <v>5</v>
@@ -3928,25 +3937,25 @@
         <v>17</v>
       </c>
       <c r="G169" s="8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H169" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I169">
         <v>5</v>
       </c>
       <c r="J169">
         <f>B169</f>
-        <v>2.3405797101449274E-3</v>
+        <v>2.261718102541901E-3</v>
       </c>
       <c r="K169" s="6">
         <f>0.11*(B162/B165)/46/(1-B160)</f>
-        <v>2.080515297906602E-3</v>
+        <v>2.0230388022607075E-3</v>
       </c>
       <c r="L169" s="6">
         <f>0.11*(B162/B164)/46/(1-B161)</f>
-        <v>2.6924315619967797E-3</v>
+        <v>2.5761855529249592E-3</v>
       </c>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.2">
@@ -3955,7 +3964,7 @@
       </c>
       <c r="B170" s="11">
         <f>1/B156</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="C170" t="s">
         <v>19</v>
@@ -3970,22 +3979,22 @@
         <v>43</v>
       </c>
       <c r="H170" t="s">
-        <v>119</v>
+        <v>195</v>
       </c>
       <c r="I170">
         <v>5</v>
       </c>
       <c r="J170" s="11">
         <f>B170</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="K170" s="11">
         <f>1/B158</f>
-        <v>6.1728395061728393E-12</v>
+        <v>6.0023081078426567E-12</v>
       </c>
       <c r="L170" s="11">
         <f>1/B157</f>
-        <v>6.5359477124183003E-12</v>
+        <v>6.25375749900866E-12</v>
       </c>
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.2">
@@ -3994,7 +4003,7 @@
       </c>
       <c r="B171" s="11">
         <f>1/B156</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="C171" t="s">
         <v>19</v>
@@ -4009,22 +4018,22 @@
         <v>49</v>
       </c>
       <c r="H171" t="s">
-        <v>119</v>
+        <v>195</v>
       </c>
       <c r="I171">
         <v>5</v>
       </c>
       <c r="J171" s="11">
         <f>B171</f>
-        <v>6.313131313131313E-12</v>
+        <v>6.1004217513912804E-12</v>
       </c>
       <c r="K171" s="11">
         <f>1/B158</f>
-        <v>6.1728395061728393E-12</v>
+        <v>6.0023081078426567E-12</v>
       </c>
       <c r="L171" s="11">
         <f>1/B157</f>
-        <v>6.5359477124183003E-12</v>
+        <v>6.25375749900866E-12</v>
       </c>
     </row>
     <row r="172" spans="1:12" x14ac:dyDescent="0.2">
@@ -4053,11 +4062,11 @@
     </row>
     <row r="173" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B173" s="12">
         <f>B169*3</f>
-        <v>7.0217391304347818E-3</v>
+        <v>6.7851543076257025E-3</v>
       </c>
       <c r="D173" t="s">
         <v>23</v>
@@ -4069,31 +4078,31 @@
         <v>20</v>
       </c>
       <c r="H173" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I173">
         <v>5</v>
       </c>
       <c r="J173" s="6">
         <f>B173</f>
-        <v>7.0217391304347818E-3</v>
+        <v>6.7851543076257025E-3</v>
       </c>
       <c r="K173" s="6">
         <f>K169*3</f>
-        <v>6.2415458937198059E-3</v>
+        <v>6.069116406782123E-3</v>
       </c>
       <c r="L173" s="6">
         <f>L169*3</f>
-        <v>8.0772946859903397E-3</v>
+        <v>7.7285566587748777E-3</v>
       </c>
     </row>
     <row r="174" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B174" s="11">
         <f>0.00186*(B169*46*B163/3.6)</f>
-        <v>2.7447916666666669E-5</v>
+        <v>2.6523108669611446E-5</v>
       </c>
       <c r="D174" t="s">
         <v>23</v>
@@ -4105,22 +4114,22 @@
         <v>20</v>
       </c>
       <c r="H174" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I174">
         <v>5</v>
       </c>
       <c r="J174" s="6">
         <f t="shared" ref="J174:J180" si="6">B174</f>
-        <v>2.7447916666666669E-5</v>
+        <v>2.6523108669611446E-5</v>
       </c>
       <c r="K174" s="6">
         <f>0.00186*(B169*46*B164/3.6)</f>
-        <v>2.4703125000000002E-5</v>
+        <v>2.3870797802650298E-5</v>
       </c>
       <c r="L174" s="6">
         <f>0.00186*(B169*46*B165/3.6)</f>
-        <v>3.0192708333333338E-5</v>
+        <v>2.9175419536572591E-5</v>
       </c>
     </row>
     <row r="175" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4129,7 +4138,7 @@
       </c>
       <c r="B175">
         <f>0.00117*(B169*46*B163/3.6)</f>
-        <v>1.7265625000000001E-5</v>
+        <v>1.6683890937336232E-5</v>
       </c>
       <c r="D175" t="s">
         <v>23</v>
@@ -4141,31 +4150,31 @@
         <v>20</v>
       </c>
       <c r="H175" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I175">
         <v>5</v>
       </c>
       <c r="J175" s="6">
         <f t="shared" si="6"/>
-        <v>1.7265625000000001E-5</v>
+        <v>1.6683890937336232E-5</v>
       </c>
       <c r="K175" s="6">
         <f>0.00117*(B169*46*B164/3.6)</f>
-        <v>1.5539062499999999E-5</v>
+        <v>1.5015501843602608E-5</v>
       </c>
       <c r="L175" s="6">
         <f>0.00117*(B169*46*B165/3.6)</f>
-        <v>1.8992187500000003E-5</v>
+        <v>1.8352280031069855E-5</v>
       </c>
     </row>
     <row r="176" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B176" s="11">
         <f>0.00003*(B169*46*B163/3.6)</f>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="D176" t="s">
         <v>23</v>
@@ -4177,31 +4186,31 @@
         <v>20</v>
       </c>
       <c r="H176" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I176">
         <v>5</v>
       </c>
       <c r="J176" s="6">
         <f t="shared" si="6"/>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="K176" s="6">
         <f>0.00003*(B169*46*B164/3.6)</f>
-        <v>3.984375E-7</v>
+        <v>3.8501286778468222E-7</v>
       </c>
       <c r="L176" s="6">
         <f>0.00003*(B169*46*B165/3.6)</f>
-        <v>4.8697916666666668E-7</v>
+        <v>4.7057128284794499E-7</v>
       </c>
     </row>
     <row r="177" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B177" s="11">
         <f>0.00003*(B169*46*B163/3.6)</f>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="D177" t="s">
         <v>23</v>
@@ -4213,31 +4222,31 @@
         <v>20</v>
       </c>
       <c r="H177" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I177">
         <v>5</v>
       </c>
       <c r="J177" s="6">
         <f t="shared" si="6"/>
-        <v>4.4270833333333331E-7</v>
+        <v>4.2779207531631361E-7</v>
       </c>
       <c r="K177" s="6">
         <f>0.00003*(B169*46*B164/3.6)</f>
-        <v>3.984375E-7</v>
+        <v>3.8501286778468222E-7</v>
       </c>
       <c r="L177" s="6">
         <f>0.00003*(B169*46*B165/3.6)</f>
-        <v>4.8697916666666668E-7</v>
+        <v>4.7057128284794499E-7</v>
       </c>
     </row>
     <row r="178" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B178" s="11">
         <f>B169*0.02</f>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="D178" t="s">
         <v>23</v>
@@ -4249,31 +4258,31 @@
         <v>20</v>
       </c>
       <c r="H178" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I178">
         <v>5</v>
       </c>
       <c r="J178" s="6">
         <f t="shared" si="6"/>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="K178" s="6">
         <f>J178</f>
-        <v>4.6811594202898551E-5</v>
+        <v>4.5234362050838021E-5</v>
       </c>
       <c r="L178" s="6">
         <f>0.067*B169</f>
-        <v>1.5681884057971014E-4</v>
+        <v>1.5153511287030737E-4</v>
       </c>
     </row>
     <row r="179" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B179" s="11">
         <f>0.00038*(B169*46*B163/3.6)</f>
-        <v>5.607638888888889E-6</v>
+        <v>5.4186996206733058E-6</v>
       </c>
       <c r="D179" t="s">
         <v>23</v>
@@ -4285,31 +4294,31 @@
         <v>20</v>
       </c>
       <c r="H179" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I179">
         <v>5</v>
       </c>
       <c r="J179" s="6">
         <f t="shared" si="6"/>
-        <v>5.607638888888889E-6</v>
+        <v>5.4186996206733058E-6</v>
       </c>
       <c r="K179" s="6">
         <f>0.00038*(B169*46*B164/3.6)</f>
-        <v>5.0468749999999999E-6</v>
+        <v>4.8768296586059753E-6</v>
       </c>
       <c r="L179" s="6">
         <f>0.00038*(B169*46*B165/3.6)</f>
-        <v>6.168402777777779E-6</v>
+        <v>5.9605695827406364E-6</v>
       </c>
     </row>
     <row r="180" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B180" s="11">
         <f>0.00002*(B169*46*B163/3.6)</f>
-        <v>2.9513888888888889E-7</v>
+        <v>2.8519471687754242E-7</v>
       </c>
       <c r="D180" t="s">
         <v>23</v>
@@ -4321,22 +4330,22 @@
         <v>20</v>
       </c>
       <c r="H180" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I180">
         <v>5</v>
       </c>
       <c r="J180" s="6">
         <f t="shared" si="6"/>
-        <v>2.9513888888888889E-7</v>
+        <v>2.8519471687754242E-7</v>
       </c>
       <c r="K180" s="11">
         <f>0.00002*(B169*46*B164/3.6)</f>
-        <v>2.65625E-7</v>
+        <v>2.5667524518978816E-7</v>
       </c>
       <c r="L180">
         <f>0.00002*(B169*46*B165/3.6)</f>
-        <v>3.2465277777777784E-7</v>
+        <v>3.1371418856529668E-7</v>
       </c>
     </row>
     <row r="182" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -4344,7 +4353,7 @@
         <v>3</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.2">
@@ -4352,7 +4361,7 @@
         <v>11</v>
       </c>
       <c r="B183" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.2">
@@ -4360,7 +4369,7 @@
         <v>10</v>
       </c>
       <c r="B184" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.2">
@@ -4389,7 +4398,7 @@
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B188" s="11">
         <f>parameters!N4</f>
@@ -4398,7 +4407,7 @@
     </row>
     <row r="189" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B189" s="11">
         <f>parameters!O4</f>
@@ -4407,7 +4416,7 @@
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B190" s="11">
         <f>parameters!P4</f>
@@ -4416,7 +4425,7 @@
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B191" s="13">
         <v>0</v>
@@ -4424,7 +4433,7 @@
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B192" s="13">
         <v>0</v>
@@ -4432,7 +4441,7 @@
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B193" s="13">
         <v>0</v>
@@ -4440,7 +4449,7 @@
     </row>
     <row r="194" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B194" s="13">
         <f>parameters!$C$15</f>
@@ -4449,7 +4458,7 @@
     </row>
     <row r="195" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B195" s="13">
         <f>parameters!C22</f>
@@ -4458,7 +4467,7 @@
     </row>
     <row r="196" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B196" s="13">
         <f>parameters!D22</f>
@@ -4467,7 +4476,7 @@
     </row>
     <row r="197" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B197" s="13">
         <f>parameters!E22</f>
@@ -4542,14 +4551,14 @@
     </row>
     <row r="201" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B201" s="12">
         <f>0.11*(B194/B195)/46/(1-B191)</f>
         <v>2.0151056763285029E-3</v>
       </c>
       <c r="C201" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E201" t="s">
         <v>9</v>
@@ -4558,10 +4567,10 @@
         <v>17</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="H201" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I201">
         <v>5</v>
@@ -4600,7 +4609,7 @@
         <v>43</v>
       </c>
       <c r="H202" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J202" s="11"/>
       <c r="K202" s="11"/>
@@ -4627,7 +4636,7 @@
         <v>49</v>
       </c>
       <c r="H203" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="J203" s="11"/>
       <c r="K203" s="11"/>
@@ -4659,7 +4668,7 @@
     </row>
     <row r="205" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B205" s="12">
         <f>B201*3.15</f>
@@ -4675,7 +4684,7 @@
         <v>20</v>
       </c>
       <c r="H205" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I205">
         <v>5</v>
@@ -4695,7 +4704,7 @@
     </row>
     <row r="206" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B206" s="11">
         <f>0.0009*(B201*43*B195/3.6)</f>
@@ -4711,7 +4720,7 @@
         <v>20</v>
       </c>
       <c r="H206" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I206">
         <v>5</v>
@@ -4747,7 +4756,7 @@
         <v>20</v>
       </c>
       <c r="H207" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I207">
         <v>5</v>
@@ -4767,7 +4776,7 @@
     </row>
     <row r="208" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B208" s="11">
         <f>0.0000163*0.2</f>
@@ -4783,7 +4792,7 @@
         <v>20</v>
       </c>
       <c r="H208" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I208">
         <v>5</v>
@@ -4803,7 +4812,7 @@
     </row>
     <row r="209" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B209" s="11">
         <f>0.00001*(B201*43*B195/3.6)</f>
@@ -4819,7 +4828,7 @@
         <v>20</v>
       </c>
       <c r="H209" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I209">
         <v>5</v>
@@ -4839,7 +4848,7 @@
     </row>
     <row r="210" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B210" s="11">
         <f>0.00041*(B201*43*B195/3.6)</f>
@@ -4855,7 +4864,7 @@
         <v>20</v>
       </c>
       <c r="H210" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I210">
         <v>5</v>
@@ -4875,7 +4884,7 @@
     </row>
     <row r="211" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B211" s="11">
         <f>0.00003*(B201*43*B195/3.6)</f>
@@ -4891,7 +4900,7 @@
         <v>20</v>
       </c>
       <c r="H211" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I211">
         <v>5</v>
@@ -4914,7 +4923,7 @@
         <v>3</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="214" spans="1:12" x14ac:dyDescent="0.2">
@@ -4922,7 +4931,7 @@
         <v>11</v>
       </c>
       <c r="B214" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="215" spans="1:12" x14ac:dyDescent="0.2">
@@ -4930,7 +4939,7 @@
         <v>10</v>
       </c>
       <c r="B215" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="216" spans="1:12" x14ac:dyDescent="0.2">
@@ -4959,7 +4968,7 @@
     </row>
     <row r="219" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B219" s="11">
         <f>parameters!N4</f>
@@ -4968,7 +4977,7 @@
     </row>
     <row r="220" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B220" s="11">
         <f>parameters!O4</f>
@@ -4977,7 +4986,7 @@
     </row>
     <row r="221" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B221" s="11">
         <f>parameters!P4</f>
@@ -4986,7 +4995,7 @@
     </row>
     <row r="222" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B222" s="13">
         <f>parameters!I41</f>
@@ -4995,7 +5004,7 @@
     </row>
     <row r="223" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B223" s="13">
         <f>parameters!J41</f>
@@ -5004,7 +5013,7 @@
     </row>
     <row r="224" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B224" s="13">
         <f>parameters!K41</f>
@@ -5013,7 +5022,7 @@
     </row>
     <row r="225" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B225" s="13">
         <f>parameters!$C$15</f>
@@ -5022,7 +5031,7 @@
     </row>
     <row r="226" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B226" s="13">
         <f>parameters!C22</f>
@@ -5031,7 +5040,7 @@
     </row>
     <row r="227" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B227" s="13">
         <f>parameters!D22</f>
@@ -5040,7 +5049,7 @@
     </row>
     <row r="228" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B228" s="13">
         <f>parameters!E22</f>
@@ -5115,7 +5124,7 @@
     </row>
     <row r="232" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>168</v>
+        <v>196</v>
       </c>
       <c r="B232" s="12">
         <f>0.11*(B225/B226)/46/(1-B222)</f>
@@ -5131,10 +5140,10 @@
         <v>17</v>
       </c>
       <c r="G232" s="8" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="H232" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I232">
         <v>5</v>
@@ -5173,7 +5182,7 @@
         <v>43</v>
       </c>
       <c r="H233" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J233" s="11"/>
       <c r="K233" s="11"/>
@@ -5200,7 +5209,7 @@
         <v>49</v>
       </c>
       <c r="H234" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J234" s="11"/>
       <c r="K234" s="11"/>
@@ -5232,7 +5241,7 @@
     </row>
     <row r="236" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B236" s="12">
         <f>B232*3.15</f>
@@ -5248,7 +5257,7 @@
         <v>20</v>
       </c>
       <c r="H236" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I236">
         <v>5</v>
@@ -5268,7 +5277,7 @@
     </row>
     <row r="237" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B237" s="11">
         <f>0.0009*(B232*43*B226/3.6)</f>
@@ -5284,7 +5293,7 @@
         <v>20</v>
       </c>
       <c r="H237" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I237">
         <v>5</v>
@@ -5320,7 +5329,7 @@
         <v>20</v>
       </c>
       <c r="H238" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I238">
         <v>5</v>
@@ -5340,7 +5349,7 @@
     </row>
     <row r="239" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B239" s="11">
         <f>0.0000163*0.2</f>
@@ -5356,7 +5365,7 @@
         <v>20</v>
       </c>
       <c r="H239" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I239">
         <v>5</v>
@@ -5376,7 +5385,7 @@
     </row>
     <row r="240" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B240" s="11">
         <f>0.00001*(B232*43*B226/3.6)</f>
@@ -5392,7 +5401,7 @@
         <v>20</v>
       </c>
       <c r="H240" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I240">
         <v>5</v>
@@ -5412,7 +5421,7 @@
     </row>
     <row r="241" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B241" s="11">
         <f>0.00041*(B232*43*B226/3.6)</f>
@@ -5428,7 +5437,7 @@
         <v>20</v>
       </c>
       <c r="H241" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I241">
         <v>5</v>
@@ -5448,7 +5457,7 @@
     </row>
     <row r="242" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B242" s="11">
         <f>0.00003*(B232*43*B226/3.6)</f>
@@ -5464,7 +5473,7 @@
         <v>20</v>
       </c>
       <c r="H242" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I242">
         <v>5</v>
@@ -5487,7 +5496,7 @@
         <v>3</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="245" spans="1:12" x14ac:dyDescent="0.2">
@@ -5495,7 +5504,7 @@
         <v>11</v>
       </c>
       <c r="B245" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="246" spans="1:12" x14ac:dyDescent="0.2">
@@ -5503,7 +5512,7 @@
         <v>10</v>
       </c>
       <c r="B246" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="247" spans="1:12" x14ac:dyDescent="0.2">
@@ -5532,7 +5541,7 @@
     </row>
     <row r="250" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B250" s="11">
         <f>parameters!N4</f>
@@ -5541,7 +5550,7 @@
     </row>
     <row r="251" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B251" s="11">
         <f>parameters!O4</f>
@@ -5550,7 +5559,7 @@
     </row>
     <row r="252" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B252" s="11">
         <f>parameters!P4</f>
@@ -5559,7 +5568,7 @@
     </row>
     <row r="253" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B253" s="13">
         <f>parameters!I72</f>
@@ -5568,7 +5577,7 @@
     </row>
     <row r="254" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B254" s="13">
         <f>parameters!J72</f>
@@ -5577,7 +5586,7 @@
     </row>
     <row r="255" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B255" s="13">
         <f>parameters!K72</f>
@@ -5586,7 +5595,7 @@
     </row>
     <row r="256" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B256" s="13">
         <f>parameters!$C$15</f>
@@ -5595,7 +5604,7 @@
     </row>
     <row r="257" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B257" s="13">
         <f>parameters!C22</f>
@@ -5604,7 +5613,7 @@
     </row>
     <row r="258" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B258" s="13">
         <f>parameters!D22</f>
@@ -5613,7 +5622,7 @@
     </row>
     <row r="259" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B259" s="13">
         <f>parameters!E22</f>
@@ -5688,7 +5697,7 @@
     </row>
     <row r="263" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B263" s="12">
         <f>0.11*(B256/B257)/46/(1-B253)</f>
@@ -5704,10 +5713,10 @@
         <v>17</v>
       </c>
       <c r="G263" s="8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H263" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I263">
         <v>5</v>
@@ -5746,7 +5755,7 @@
         <v>43</v>
       </c>
       <c r="H264" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J264" s="11"/>
       <c r="K264" s="11"/>
@@ -5773,7 +5782,7 @@
         <v>49</v>
       </c>
       <c r="H265" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J265" s="11"/>
       <c r="K265" s="11"/>
@@ -5805,7 +5814,7 @@
     </row>
     <row r="267" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B267" s="12">
         <f>B263*3.15</f>
@@ -5821,7 +5830,7 @@
         <v>20</v>
       </c>
       <c r="H267" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I267">
         <v>5</v>
@@ -5841,7 +5850,7 @@
     </row>
     <row r="268" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B268" s="11">
         <f>0.0009*(B263*43*B257/3.6)</f>
@@ -5857,7 +5866,7 @@
         <v>20</v>
       </c>
       <c r="H268" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I268">
         <v>5</v>
@@ -5893,7 +5902,7 @@
         <v>20</v>
       </c>
       <c r="H269" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I269">
         <v>5</v>
@@ -5913,7 +5922,7 @@
     </row>
     <row r="270" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B270" s="11">
         <f>0.0000163*0.2</f>
@@ -5929,7 +5938,7 @@
         <v>20</v>
       </c>
       <c r="H270" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I270">
         <v>5</v>
@@ -5949,7 +5958,7 @@
     </row>
     <row r="271" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B271" s="11">
         <f>0.00001*(B263*43*B257/3.6)</f>
@@ -5965,7 +5974,7 @@
         <v>20</v>
       </c>
       <c r="H271" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I271">
         <v>5</v>
@@ -5985,7 +5994,7 @@
     </row>
     <row r="272" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B272" s="11">
         <f>0.00041*(B263*43*B257/3.6)</f>
@@ -6001,7 +6010,7 @@
         <v>20</v>
       </c>
       <c r="H272" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I272">
         <v>5</v>
@@ -6021,7 +6030,7 @@
     </row>
     <row r="273" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B273" s="11">
         <f>0.00003*(B263*43*B257/3.6)</f>
@@ -6037,7 +6046,7 @@
         <v>20</v>
       </c>
       <c r="H273" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="I273">
         <v>5</v>
@@ -6064,7 +6073,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95F1A7F4-A2B5-7747-AA61-2990069064F9}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.1640625" bestFit="1" customWidth="1"/>
@@ -6087,62 +6096,62 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="E3" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="I3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="L3" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="M3" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D4" s="16">
         <v>1</v>
@@ -6186,23 +6195,23 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="16">
         <v>0.43880000000000002</v>
       </c>
       <c r="E5" s="16">
-        <f t="shared" ref="E5:E10" si="0">1/D5</f>
+        <f t="shared" ref="E5:E11" si="0">1/D5</f>
         <v>2.2789425706472195</v>
       </c>
       <c r="F5" s="16">
         <v>1.1000000000000001</v>
       </c>
       <c r="G5" s="16">
-        <f t="shared" ref="G5:G10" si="1">E5*F5</f>
+        <f t="shared" ref="G5:G11" si="1">E5*F5</f>
         <v>2.5068368277119415</v>
       </c>
       <c r="H5" s="14">
@@ -6240,10 +6249,10 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D6" s="16">
         <v>0.35270000000000001</v>
@@ -6294,10 +6303,10 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D7" s="16">
         <v>0.25</v>
@@ -6348,10 +6357,10 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D8" s="16">
         <v>8.3300000000000006E-3</v>
@@ -6402,10 +6411,10 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D9" s="16">
         <v>0.61109999999999998</v>
@@ -6422,7 +6431,7 @@
         <v>1.8000327278677795</v>
       </c>
       <c r="H9" s="14">
-        <f t="shared" si="2"/>
+        <f>1-(1/G9)</f>
         <v>0.44445454545454544</v>
       </c>
       <c r="I9" s="13">
@@ -6455,10 +6464,10 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D10" s="16">
         <v>0.27700000000000002</v>
@@ -6506,26 +6515,83 @@
         <v>117000000000</v>
       </c>
     </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>193</v>
+      </c>
+      <c r="C11" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="16">
+        <f>26.5/36</f>
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="E11" s="16">
+        <f t="shared" si="0"/>
+        <v>1.3584905660377358</v>
+      </c>
+      <c r="F11" s="16">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G11" s="16">
+        <f t="shared" si="1"/>
+        <v>1.4943396226415095</v>
+      </c>
+      <c r="H11" s="14">
+        <f>1-(1/G11)</f>
+        <v>0.33080808080808088</v>
+      </c>
+      <c r="I11" s="13">
+        <f>I9*H11/H9</f>
+        <v>8.9316151905638519E-2</v>
+      </c>
+      <c r="J11" s="13">
+        <f>J9*H11/H9</f>
+        <v>7.4430126588032122E-2</v>
+      </c>
+      <c r="K11" s="13">
+        <f>K9*H11/H9</f>
+        <v>0.11164518988204816</v>
+      </c>
+      <c r="L11" s="15">
+        <v>7200000000</v>
+      </c>
+      <c r="M11">
+        <v>25</v>
+      </c>
+      <c r="N11" s="15">
+        <f t="shared" ref="N11" si="8">L11*M11*(1-I11)</f>
+        <v>163923092656.98508</v>
+      </c>
+      <c r="O11" s="15">
+        <f t="shared" ref="O11" si="9">L11*M11*(1-K11)</f>
+        <v>159903865821.23132</v>
+      </c>
+      <c r="P11" s="15">
+        <f t="shared" ref="P11" si="10">L11*M11*(1-J11)</f>
+        <v>166602577214.15421</v>
+      </c>
+    </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="O12" s="11"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C15" s="14">
         <f>AVERAGE(D15:E15)</f>
@@ -6540,7 +6606,7 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C16" s="14">
         <f>3.6/(0.414*19.9)</f>
@@ -6557,7 +6623,7 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C17" s="14">
         <f>3.6/(0.435*18.8)</f>
@@ -6572,7 +6638,7 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C18" s="14">
         <f>AVERAGE(D18:E18)</f>
@@ -6587,7 +6653,7 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C19" s="14">
         <f>AVERAGE(D19:E19)</f>
@@ -6602,7 +6668,7 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C20" s="14">
         <f>3.6/(0.152*48)</f>
@@ -6619,7 +6685,7 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C21" s="14">
         <f>3.6/(0.152*48)</f>
@@ -6636,7 +6702,7 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C22" s="14">
         <f>3.6/(0.166*43)</f>
@@ -6653,7 +6719,24 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>183</v>
+        <v>193</v>
+      </c>
+      <c r="C23" s="14">
+        <f>3.6/(0.152*48)</f>
+        <v>0.49342105263157898</v>
+      </c>
+      <c r="D23" s="14">
+        <f>C23*0.9</f>
+        <v>0.44407894736842107</v>
+      </c>
+      <c r="E23" s="14">
+        <f>C23*1.1</f>
+        <v>0.54276315789473695</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>